<commit_message>
Changed a few things in the experiment.py and set default temperature to 1 across the system
</commit_message>
<xml_diff>
--- a/orchestrator/experiments/aime24_results.xlsx
+++ b/orchestrator/experiments/aime24_results.xlsx
@@ -413,139 +413,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>problems</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>use_cachesaver</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>accuracy</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>prompt_tokens_used_orc</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>input_cost_orc ($)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>completion_tokens_used_orc</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>output_cost_orc ($)</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>total_cost_orc ($)</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>prompt_tokens_used_agents</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>input_cost_agents ($)</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>completion_tokens_used_agents</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>output_cost_agents ($)</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>total_cost_agents ($)</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>api_calls_orc</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>api_calls_agents</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>runtime (s)</t>
-        </is>
+      <c r="A1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="b">
+    </row>
+    <row r="3">
+      <c r="A3" t="b">
         <v>0</v>
       </c>
-      <c r="C2" t="n">
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="n">
-        <v>4487</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.00049357</v>
-      </c>
-      <c r="F2" t="n">
-        <v>498</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.00016932</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.0006628900000000001</v>
-      </c>
-      <c r="I2" t="n">
-        <v>12753</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.00140283</v>
-      </c>
-      <c r="K2" t="n">
-        <v>5995</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.0020383</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.00344113</v>
-      </c>
-      <c r="N2" t="n">
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4479</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>0.00022395</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>0.0001072</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>0.00033115</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>4363</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>0.00021815</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>18885</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>0.007554</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>0.00777215</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
         <v>1</v>
       </c>
-      <c r="O2" t="n">
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
         <v>11</v>
       </c>
-      <c r="P2" t="n">
-        <v>35.65</v>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>164.32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed the timeout limit to 300 seconds and fixed a bug in remote_orchestrator.py
</commit_message>
<xml_diff>
--- a/orchestrator/experiments/aime24_results.xlsx
+++ b/orchestrator/experiments/aime24_results.xlsx
@@ -413,92 +413,172 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="n">
+      <c r="B1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>problems</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="b">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>use_cachesaver</t>
+        </is>
+      </c>
+      <c r="B3" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>prompt_tokens_used_orc</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>4479</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>0.00022395</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>input_cost_orc ($)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.0004926899999999999</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>268</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>completion_tokens_used_orc</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>774</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>0.0001072</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>output_cost_orc ($)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.00026316</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>0.00033115</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>total_cost_orc ($)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.00075585</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>4363</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>prompt_tokens_used_agents</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>12054</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>0.00021815</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>input_cost_agents ($)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.00132594</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>18885</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>completion_tokens_used_agents</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>6767</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>0.007554</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>output_cost_agents ($)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.00230078</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>0.00777215</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>total_cost_agents ($)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.00362672</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>api_calls_orc</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>api_calls_agents</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
-        <v>164.32</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>runtime (s)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>47.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added local copy of CacheSaver
</commit_message>
<xml_diff>
--- a/orchestrator/experiments/aime24_results.xlsx
+++ b/orchestrator/experiments/aime24_results.xlsx
@@ -448,7 +448,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>774</v>
+        <v>683</v>
       </c>
     </row>
     <row r="8">
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.00026316</v>
+        <v>0.00023222</v>
       </c>
     </row>
     <row r="9">
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.00075585</v>
+        <v>0.0007249099999999999</v>
       </c>
     </row>
     <row r="10">
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>12054</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="11">
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.00132594</v>
+        <v>0.00014707</v>
       </c>
     </row>
     <row r="12">
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6767</v>
+        <v>933</v>
       </c>
     </row>
     <row r="13">
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.00230078</v>
+        <v>0.00031722</v>
       </c>
     </row>
     <row r="14">
@@ -548,7 +548,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.00362672</v>
+        <v>0.00046429</v>
       </c>
     </row>
     <row r="15">
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>47.44</v>
+        <v>29.63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>